<commit_message>
Rincian per tipe: tombol tampilkan/sembunyikan; data contoh Naragriya pakai Vasa/Nava
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Y8Us56muFbCjBwSqpr5Hk
</commit_message>
<xml_diff>
--- a/REKAP_ALL_TIME_DUMMY.xlsx
+++ b/REKAP_ALL_TIME_DUMMY.xlsx
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>NARA Standard</t>
+          <t>VASA Standard</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>7 x 15</t>
+          <t>5 x 14</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>NARA Standard</t>
+          <t>NAVA Standard</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>7 x 15</t>
+          <t>5 x 15</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>NARA Hook</t>
+          <t>NAVA Hook</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>8 x 16</t>
+          <t>5 x 18</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>NARA Standard</t>
+          <t>VASA Standard</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -5181,7 +5181,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>7 x 15</t>
+          <t>5 x 14</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>NARA Standard</t>
+          <t>NAVA Standard</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>7 x 15</t>
+          <t>5 x 15</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -6931,7 +6931,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>NARA Hook</t>
+          <t>NAVA Hook</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -6941,7 +6941,7 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>8 x 16</t>
+          <t>5 x 18</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -8603,7 +8603,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>NARA Standard</t>
+          <t>VASA Standard</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -8613,7 +8613,7 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>7 x 15</t>
+          <t>5 x 14</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>NARA Standard</t>
+          <t>NAVA Standard</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -9317,7 +9317,7 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>7 x 15</t>
+          <t>5 x 15</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Data contoh: harga dibuat berpola supaya jelas dummy, rentang tetap sesuai segmen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Y8Us56muFbCjBwSqpr5Hk
</commit_message>
<xml_diff>
--- a/REKAP_ALL_TIME_DUMMY.xlsx
+++ b/REKAP_ALL_TIME_DUMMY.xlsx
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>1.063</v>
+        <v>1.111</v>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>4.772</v>
+        <v>3.21</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="M4" s="6" t="n">
-        <v>3.003</v>
+        <v>3</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="M5" s="6" t="n">
-        <v>3.068</v>
+        <v>3.111</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="M6" s="6" t="n">
-        <v>1.093</v>
+        <v>1.001</v>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1.926</v>
+        <v>2</v>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
         </is>
       </c>
       <c r="M9" s="6" t="n">
-        <v>6.273</v>
+        <v>5.432</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="M10" s="6" t="n">
-        <v>1.232</v>
+        <v>1.202</v>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="M11" s="6" t="n">
-        <v>2.24</v>
+        <v>2.222</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="M12" s="6" t="n">
-        <v>1.016</v>
+        <v>1.101</v>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="M13" s="6" t="n">
-        <v>1.705</v>
+        <v>1.717</v>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="M14" s="6" t="n">
-        <v>3.345</v>
+        <v>3.333</v>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="M15" s="6" t="n">
-        <v>1.554</v>
+        <v>1.555</v>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="M16" s="6" t="n">
-        <v>1.41</v>
+        <v>1.234</v>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         </is>
       </c>
       <c r="M17" s="6" t="n">
-        <v>1.791</v>
+        <v>1.771</v>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="M18" s="6" t="n">
-        <v>3.507</v>
+        <v>4.567</v>
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
@@ -2231,7 +2231,7 @@
         </is>
       </c>
       <c r="M19" s="6" t="n">
-        <v>2.863</v>
+        <v>2.777</v>
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
@@ -2319,7 +2319,7 @@
         </is>
       </c>
       <c r="M20" s="6" t="n">
-        <v>2.835</v>
+        <v>2.727</v>
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="M21" s="6" t="n">
-        <v>1.626</v>
+        <v>1.313</v>
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="M23" s="6" t="n">
-        <v>0.946</v>
+        <v>0.987</v>
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="M24" s="6" t="n">
-        <v>2.715</v>
+        <v>2.828</v>
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
@@ -2759,7 +2759,7 @@
         </is>
       </c>
       <c r="M25" s="6" t="n">
-        <v>4.733</v>
+        <v>3.456</v>
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="M26" s="6" t="n">
-        <v>1.628</v>
+        <v>1.515</v>
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
         </is>
       </c>
       <c r="M27" s="6" t="n">
-        <v>1.642</v>
+        <v>1.616</v>
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
         </is>
       </c>
       <c r="M28" s="6" t="n">
-        <v>4.433</v>
+        <v>3.567</v>
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
         </is>
       </c>
       <c r="M29" s="6" t="n">
-        <v>1.397</v>
+        <v>1.333</v>
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="M30" s="6" t="n">
-        <v>1.616</v>
+        <v>1.551</v>
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="M31" s="6" t="n">
-        <v>1.042</v>
+        <v>1.123</v>
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
@@ -3375,7 +3375,7 @@
         </is>
       </c>
       <c r="M32" s="6" t="n">
-        <v>1.39</v>
+        <v>1.414</v>
       </c>
       <c r="N32" s="3" t="inlineStr">
         <is>
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="M33" s="6" t="n">
-        <v>1.855</v>
+        <v>1.414</v>
       </c>
       <c r="N33" s="3" t="inlineStr">
         <is>
@@ -3551,7 +3551,7 @@
         </is>
       </c>
       <c r="M34" s="6" t="n">
-        <v>5.024</v>
+        <v>3.321</v>
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="M35" s="6" t="n">
-        <v>1.096</v>
+        <v>1.1</v>
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="M36" s="6" t="n">
-        <v>2.98</v>
+        <v>3.003</v>
       </c>
       <c r="N36" s="3" t="inlineStr">
         <is>
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="M37" s="6" t="n">
-        <v>3.037</v>
+        <v>3.131</v>
       </c>
       <c r="N37" s="3" t="inlineStr">
         <is>
@@ -3903,7 +3903,7 @@
         </is>
       </c>
       <c r="M38" s="6" t="n">
-        <v>1.551</v>
+        <v>1.565</v>
       </c>
       <c r="N38" s="3" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="M39" s="6" t="n">
-        <v>2.968</v>
+        <v>3.033</v>
       </c>
       <c r="N39" s="3" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
         </is>
       </c>
       <c r="M40" s="6" t="n">
-        <v>3.188</v>
+        <v>3.113</v>
       </c>
       <c r="N40" s="3" t="inlineStr">
         <is>
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="M41" s="6" t="n">
-        <v>1.065</v>
+        <v>1.111</v>
       </c>
       <c r="N41" s="3" t="inlineStr">
         <is>
@@ -4255,7 +4255,7 @@
         </is>
       </c>
       <c r="M42" s="6" t="n">
-        <v>2.172</v>
+        <v>2.002</v>
       </c>
       <c r="N42" s="3" t="inlineStr">
         <is>
@@ -4343,7 +4343,7 @@
         </is>
       </c>
       <c r="M43" s="6" t="n">
-        <v>3.44</v>
+        <v>3.434</v>
       </c>
       <c r="N43" s="3" t="inlineStr">
         <is>
@@ -4431,7 +4431,7 @@
         </is>
       </c>
       <c r="M44" s="6" t="n">
-        <v>1.232</v>
+        <v>1.212</v>
       </c>
       <c r="N44" s="3" t="inlineStr">
         <is>
@@ -4519,7 +4519,7 @@
         </is>
       </c>
       <c r="M45" s="6" t="n">
-        <v>1.665</v>
+        <v>1.818</v>
       </c>
       <c r="N45" s="3" t="inlineStr">
         <is>
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="M46" s="6" t="n">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="N46" s="3" t="inlineStr">
         <is>
@@ -4695,7 +4695,7 @@
         </is>
       </c>
       <c r="M47" s="6" t="n">
-        <v>4.761</v>
+        <v>3.678</v>
       </c>
       <c r="N47" s="3" t="inlineStr">
         <is>
@@ -4783,7 +4783,7 @@
         </is>
       </c>
       <c r="M48" s="6" t="n">
-        <v>1.082</v>
+        <v>1.001</v>
       </c>
       <c r="N48" s="3" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="M49" s="6" t="n">
-        <v>2.681</v>
+        <v>2.626</v>
       </c>
       <c r="N49" s="3" t="inlineStr">
         <is>
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="M50" s="6" t="n">
-        <v>8.493</v>
+        <v>6.789</v>
       </c>
       <c r="N50" s="3" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         </is>
       </c>
       <c r="M51" s="6" t="n">
-        <v>1.447</v>
+        <v>1.212</v>
       </c>
       <c r="N51" s="3" t="inlineStr">
         <is>
@@ -5135,7 +5135,7 @@
         </is>
       </c>
       <c r="M52" s="6" t="n">
-        <v>1.868</v>
+        <v>1.881</v>
       </c>
       <c r="N52" s="3" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
         </is>
       </c>
       <c r="M53" s="6" t="n">
-        <v>2.745</v>
+        <v>2.707</v>
       </c>
       <c r="N53" s="3" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
         </is>
       </c>
       <c r="M54" s="6" t="n">
-        <v>1.635</v>
+        <v>1.661</v>
       </c>
       <c r="N54" s="3" t="inlineStr">
         <is>
@@ -5399,7 +5399,7 @@
         </is>
       </c>
       <c r="M55" s="6" t="n">
-        <v>1.876</v>
+        <v>1.888</v>
       </c>
       <c r="N55" s="3" t="inlineStr">
         <is>
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="M56" s="6" t="n">
-        <v>6.667</v>
+        <v>5.678</v>
       </c>
       <c r="N56" s="3" t="inlineStr">
         <is>
@@ -5575,7 +5575,7 @@
         </is>
       </c>
       <c r="M57" s="6" t="n">
-        <v>1.771</v>
+        <v>1.678</v>
       </c>
       <c r="N57" s="3" t="inlineStr">
         <is>
@@ -5663,7 +5663,7 @@
         </is>
       </c>
       <c r="M58" s="6" t="n">
-        <v>1.566</v>
+        <v>1.331</v>
       </c>
       <c r="N58" s="3" t="inlineStr">
         <is>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="M59" s="6" t="n">
-        <v>2.792</v>
+        <v>2.772</v>
       </c>
       <c r="N59" s="3" t="inlineStr">
         <is>
@@ -5839,7 +5839,7 @@
         </is>
       </c>
       <c r="M60" s="6" t="n">
-        <v>1.179</v>
+        <v>1.101</v>
       </c>
       <c r="N60" s="3" t="inlineStr">
         <is>
@@ -5927,7 +5927,7 @@
         </is>
       </c>
       <c r="M61" s="6" t="n">
-        <v>1.604</v>
+        <v>1.333</v>
       </c>
       <c r="N61" s="3" t="inlineStr">
         <is>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="M62" s="6" t="n">
-        <v>4.289</v>
+        <v>4.321</v>
       </c>
       <c r="N62" s="3" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         </is>
       </c>
       <c r="M63" s="6" t="n">
-        <v>2.26</v>
+        <v>2.332</v>
       </c>
       <c r="N63" s="3" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         </is>
       </c>
       <c r="M64" s="6" t="n">
-        <v>1.89</v>
+        <v>1.441</v>
       </c>
       <c r="N64" s="3" t="inlineStr">
         <is>
@@ -6279,7 +6279,7 @@
         </is>
       </c>
       <c r="M65" s="6" t="n">
-        <v>1.574</v>
+        <v>1.221</v>
       </c>
       <c r="N65" s="3" t="inlineStr">
         <is>
@@ -6367,7 +6367,7 @@
         </is>
       </c>
       <c r="M66" s="6" t="n">
-        <v>2.76</v>
+        <v>2.882</v>
       </c>
       <c r="N66" s="3" t="inlineStr">
         <is>
@@ -6455,7 +6455,7 @@
         </is>
       </c>
       <c r="M67" s="6" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="N67" s="3" t="inlineStr">
         <is>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="M68" s="6" t="n">
-        <v>2.238</v>
+        <v>2.323</v>
       </c>
       <c r="N68" s="3" t="inlineStr">
         <is>
@@ -6631,7 +6631,7 @@
         </is>
       </c>
       <c r="M69" s="6" t="n">
-        <v>2.452</v>
+        <v>2.345</v>
       </c>
       <c r="N69" s="3" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
         </is>
       </c>
       <c r="M70" s="6" t="n">
-        <v>1.433</v>
+        <v>1.313</v>
       </c>
       <c r="N70" s="3" t="inlineStr">
         <is>
@@ -6807,7 +6807,7 @@
         </is>
       </c>
       <c r="M71" s="6" t="n">
-        <v>1.912</v>
+        <v>1.444</v>
       </c>
       <c r="N71" s="3" t="inlineStr">
         <is>
@@ -6895,7 +6895,7 @@
         </is>
       </c>
       <c r="M72" s="6" t="n">
-        <v>1.686</v>
+        <v>1.717</v>
       </c>
       <c r="N72" s="3" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="M73" s="6" t="n">
-        <v>3.04</v>
+        <v>3.03</v>
       </c>
       <c r="N73" s="3" t="inlineStr">
         <is>
@@ -7071,7 +7071,7 @@
         </is>
       </c>
       <c r="M74" s="6" t="n">
-        <v>6.045</v>
+        <v>5.555</v>
       </c>
       <c r="N74" s="3" t="inlineStr">
         <is>
@@ -7159,7 +7159,7 @@
         </is>
       </c>
       <c r="M75" s="6" t="n">
-        <v>1.742</v>
+        <v>1.777</v>
       </c>
       <c r="N75" s="3" t="inlineStr">
         <is>
@@ -7247,7 +7247,7 @@
         </is>
       </c>
       <c r="M76" s="6" t="n">
-        <v>2.308</v>
+        <v>2.222</v>
       </c>
       <c r="N76" s="3" t="inlineStr">
         <is>
@@ -7335,7 +7335,7 @@
         </is>
       </c>
       <c r="M77" s="6" t="n">
-        <v>1.091</v>
+        <v>1.011</v>
       </c>
       <c r="N77" s="3" t="inlineStr">
         <is>
@@ -7423,7 +7423,7 @@
         </is>
       </c>
       <c r="M78" s="6" t="n">
-        <v>1.086</v>
+        <v>1.123</v>
       </c>
       <c r="N78" s="3" t="inlineStr">
         <is>
@@ -7511,7 +7511,7 @@
         </is>
       </c>
       <c r="M79" s="6" t="n">
-        <v>2.777</v>
+        <v>2.662</v>
       </c>
       <c r="N79" s="3" t="inlineStr">
         <is>
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="M80" s="6" t="n">
-        <v>0.973</v>
+        <v>0.999</v>
       </c>
       <c r="N80" s="3" t="inlineStr">
         <is>
@@ -7687,7 +7687,7 @@
         </is>
       </c>
       <c r="M81" s="6" t="n">
-        <v>2.709</v>
+        <v>2.789</v>
       </c>
       <c r="N81" s="3" t="inlineStr">
         <is>
@@ -7775,7 +7775,7 @@
         </is>
       </c>
       <c r="M82" s="6" t="n">
-        <v>1.071</v>
+        <v>1.02</v>
       </c>
       <c r="N82" s="3" t="inlineStr">
         <is>
@@ -7863,7 +7863,7 @@
         </is>
       </c>
       <c r="M83" s="6" t="n">
-        <v>1.406</v>
+        <v>1.441</v>
       </c>
       <c r="N83" s="3" t="inlineStr">
         <is>
@@ -7951,7 +7951,7 @@
         </is>
       </c>
       <c r="M84" s="6" t="n">
-        <v>1.712</v>
+        <v>1.555</v>
       </c>
       <c r="N84" s="3" t="inlineStr">
         <is>
@@ -8039,7 +8039,7 @@
         </is>
       </c>
       <c r="M85" s="6" t="n">
-        <v>0.897</v>
+        <v>0.909</v>
       </c>
       <c r="N85" s="3" t="inlineStr">
         <is>
@@ -8127,7 +8127,7 @@
         </is>
       </c>
       <c r="M86" s="6" t="n">
-        <v>2.7</v>
+        <v>2.808</v>
       </c>
       <c r="N86" s="3" t="inlineStr">
         <is>
@@ -8215,7 +8215,7 @@
         </is>
       </c>
       <c r="M87" s="6" t="n">
-        <v>6.855</v>
+        <v>7.654</v>
       </c>
       <c r="N87" s="3" t="inlineStr">
         <is>
@@ -8303,7 +8303,7 @@
         </is>
       </c>
       <c r="M88" s="6" t="n">
-        <v>5.014</v>
+        <v>3.789</v>
       </c>
       <c r="N88" s="3" t="inlineStr">
         <is>
@@ -8391,7 +8391,7 @@
         </is>
       </c>
       <c r="M89" s="6" t="n">
-        <v>1.768</v>
+        <v>1.323</v>
       </c>
       <c r="N89" s="3" t="inlineStr">
         <is>
@@ -8479,7 +8479,7 @@
         </is>
       </c>
       <c r="M90" s="6" t="n">
-        <v>2.082</v>
+        <v>2.02</v>
       </c>
       <c r="N90" s="3" t="inlineStr">
         <is>
@@ -8567,7 +8567,7 @@
         </is>
       </c>
       <c r="M91" s="6" t="n">
-        <v>4.701</v>
+        <v>3.999</v>
       </c>
       <c r="N91" s="3" t="inlineStr">
         <is>
@@ -8655,7 +8655,7 @@
         </is>
       </c>
       <c r="M92" s="6" t="n">
-        <v>2.79</v>
+        <v>2.77</v>
       </c>
       <c r="N92" s="3" t="inlineStr">
         <is>
@@ -8743,7 +8743,7 @@
         </is>
       </c>
       <c r="M93" s="6" t="n">
-        <v>1.433</v>
+        <v>1.234</v>
       </c>
       <c r="N93" s="3" t="inlineStr">
         <is>
@@ -8831,7 +8831,7 @@
         </is>
       </c>
       <c r="M94" s="6" t="n">
-        <v>1.947</v>
+        <v>1.818</v>
       </c>
       <c r="N94" s="3" t="inlineStr">
         <is>
@@ -8919,7 +8919,7 @@
         </is>
       </c>
       <c r="M95" s="6" t="n">
-        <v>1.128</v>
+        <v>1.1</v>
       </c>
       <c r="N95" s="3" t="inlineStr">
         <is>
@@ -9007,7 +9007,7 @@
         </is>
       </c>
       <c r="M96" s="6" t="n">
-        <v>1.115</v>
+        <v>1.111</v>
       </c>
       <c r="N96" s="3" t="inlineStr">
         <is>
@@ -9095,7 +9095,7 @@
         </is>
       </c>
       <c r="M97" s="6" t="n">
-        <v>0.972</v>
+        <v>1.03</v>
       </c>
       <c r="N97" s="3" t="inlineStr">
         <is>
@@ -9183,7 +9183,7 @@
         </is>
       </c>
       <c r="M98" s="6" t="n">
-        <v>1.175</v>
+        <v>1.001</v>
       </c>
       <c r="N98" s="3" t="inlineStr">
         <is>
@@ -9271,7 +9271,7 @@
         </is>
       </c>
       <c r="M99" s="6" t="n">
-        <v>1.614</v>
+        <v>1.222</v>
       </c>
       <c r="N99" s="3" t="inlineStr">
         <is>
@@ -9359,7 +9359,7 @@
         </is>
       </c>
       <c r="M100" s="6" t="n">
-        <v>2.835</v>
+        <v>2.888</v>
       </c>
       <c r="N100" s="3" t="inlineStr">
         <is>
@@ -9447,7 +9447,7 @@
         </is>
       </c>
       <c r="M101" s="6" t="n">
-        <v>1.103</v>
+        <v>1.101</v>
       </c>
       <c r="N101" s="3" t="inlineStr">
         <is>
@@ -9535,7 +9535,7 @@
         </is>
       </c>
       <c r="M102" s="6" t="n">
-        <v>1.151</v>
+        <v>1.221</v>
       </c>
       <c r="N102" s="3" t="inlineStr">
         <is>
@@ -9623,7 +9623,7 @@
         </is>
       </c>
       <c r="M103" s="6" t="n">
-        <v>1.08</v>
+        <v>1</v>
       </c>
       <c r="N103" s="3" t="inlineStr">
         <is>
@@ -9711,7 +9711,7 @@
         </is>
       </c>
       <c r="M104" s="6" t="n">
-        <v>1.552</v>
+        <v>1.333</v>
       </c>
       <c r="N104" s="3" t="inlineStr">
         <is>
@@ -9799,7 +9799,7 @@
         </is>
       </c>
       <c r="M105" s="6" t="n">
-        <v>0.931</v>
+        <v>0.987</v>
       </c>
       <c r="N105" s="3" t="inlineStr">
         <is>
@@ -9887,7 +9887,7 @@
         </is>
       </c>
       <c r="M106" s="6" t="n">
-        <v>1.588</v>
+        <v>1.515</v>
       </c>
       <c r="N106" s="3" t="inlineStr">
         <is>
@@ -9975,7 +9975,7 @@
         </is>
       </c>
       <c r="M107" s="6" t="n">
-        <v>2.378</v>
+        <v>2.233</v>
       </c>
       <c r="N107" s="3" t="inlineStr">
         <is>
@@ -10063,7 +10063,7 @@
         </is>
       </c>
       <c r="M108" s="6" t="n">
-        <v>4.977</v>
+        <v>3.432</v>
       </c>
       <c r="N108" s="3" t="inlineStr">
         <is>
@@ -10151,7 +10151,7 @@
         </is>
       </c>
       <c r="M109" s="6" t="n">
-        <v>2.033</v>
+        <v>2.002</v>
       </c>
       <c r="N109" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Nama cluster dan tipe di Sales Report memakai nama samaran, mengikuti sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Y8Us56muFbCjBwSqpr5Hk
</commit_message>
<xml_diff>
--- a/REKAP_ALL_TIME_DUMMY.xlsx
+++ b/REKAP_ALL_TIME_DUMMY.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,6 +119,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -560,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R109"/>
+  <dimension ref="A1:R113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -678,12 +680,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -766,12 +768,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Darmaraja Standard</t>
+          <t>Darmawisata Standard</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -854,12 +856,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>LA PLAZA</t>
+          <t>UHUY PLAZA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>LP Standard</t>
+          <t>UHP Standard</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -942,12 +944,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>NP Standard</t>
+          <t>UP Standard</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1030,12 +1032,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1118,12 +1120,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VETRA Standard</t>
+          <t>VESPA Standard</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1206,12 +1208,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>VASA Standard</t>
+          <t>VISA Standard</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1294,12 +1296,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Wanayasa Hook</t>
+          <t>Wanabisa Hook</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1382,12 +1384,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Hook</t>
+          <t>APEGEL S Hook</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1470,12 +1472,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1558,12 +1560,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1646,12 +1648,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1734,12 +1736,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>THE PLAZA</t>
+          <t>ESTHE PLAZA</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>TP Standard</t>
+          <t>EP Standard</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1822,12 +1824,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1910,12 +1912,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1998,12 +2000,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -2086,12 +2088,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DHARMAPURI</t>
+          <t>DARIPURI</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>ARUNA EKA Standard</t>
+          <t>AROMA EKA Standard</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -2174,12 +2176,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2262,12 +2264,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2350,12 +2352,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2438,12 +2440,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2526,12 +2528,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2614,12 +2616,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>NAVA Standard</t>
+          <t>NAWAR Standard</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2702,12 +2704,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2790,12 +2792,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2878,12 +2880,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>SVARA EKA Standard</t>
+          <t>SUARA EKA Standard</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2966,12 +2968,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -3054,12 +3056,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -3142,12 +3144,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -3230,12 +3232,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -3318,12 +3320,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -3406,12 +3408,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Akasha Hook</t>
+          <t>Akasih Hook</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -3494,12 +3496,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Darmaraja Standard</t>
+          <t>Darmawisata Standard</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3582,12 +3584,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -3670,12 +3672,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>NAVA Hook</t>
+          <t>NAWAR Hook</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3758,12 +3760,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>NP Standard</t>
+          <t>UP Standard</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -3846,12 +3848,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -3934,12 +3936,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LA PLAZA</t>
+          <t>UHUY PLAZA</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>LP Standard</t>
+          <t>UHP Standard</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -4022,12 +4024,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>NP Standard</t>
+          <t>UP Standard</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -4110,12 +4112,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -4198,12 +4200,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>SVARA EKA Hook</t>
+          <t>SUARA EKA Hook</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -4286,12 +4288,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>THE PLAZA</t>
+          <t>ESTHE PLAZA</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>TP Standard</t>
+          <t>EP Standard</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -4374,12 +4376,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Hook</t>
+          <t>APEGEL S Hook</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -4462,12 +4464,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Standard</t>
+          <t>AMBYAR TRI Standard</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -4550,12 +4552,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -4638,12 +4640,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -4726,12 +4728,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -4814,12 +4816,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>VETRA Hook</t>
+          <t>VESPA Hook</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -4902,12 +4904,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>SAGARA Hook</t>
+          <t>SEGERA Hook</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -4990,12 +4992,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Akasha Standard</t>
+          <t>Akasih Standard</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -5078,12 +5080,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Standard</t>
+          <t>AMBYAR TRI Standard</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -5166,12 +5168,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>VASA Standard</t>
+          <t>VISA Standard</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -5254,12 +5256,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>SVARA EKA Standard</t>
+          <t>SUARA EKA Standard</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -5342,12 +5344,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Standard</t>
+          <t>AMBYAR TRI Standard</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -5430,12 +5432,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>SAGARA Standard</t>
+          <t>SEGERA Standard</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -5518,12 +5520,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Standard</t>
+          <t>ARENA EKA Standard</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -5606,12 +5608,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -5694,12 +5696,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -5782,12 +5784,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -5870,12 +5872,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -5958,12 +5960,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>NP Hook</t>
+          <t>UP Hook</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -6046,12 +6048,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -6134,12 +6136,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Akasha Hook</t>
+          <t>Akasih Hook</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -6222,12 +6224,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Akasha Standard</t>
+          <t>Akasih Standard</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -6310,12 +6312,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>NAVA Standard</t>
+          <t>NAWAR Standard</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -6398,12 +6400,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -6486,12 +6488,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -6574,12 +6576,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Hook</t>
+          <t>AMBYAR TRI Hook</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -6662,12 +6664,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -6750,12 +6752,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Akasha Hook</t>
+          <t>Akasih Hook</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -6838,12 +6840,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Standard</t>
+          <t>ARENA EKA Standard</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -6926,12 +6928,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>NAVA Hook</t>
+          <t>NAWAR Hook</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -7014,12 +7016,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>SAGARA Standard</t>
+          <t>SEGERA Standard</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -7102,12 +7104,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -7190,12 +7192,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Hook</t>
+          <t>AMBYAR EKA Hook</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -7278,12 +7280,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -7366,12 +7368,12 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -7454,12 +7456,12 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>VETRA Hook</t>
+          <t>VESPA Hook</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -7542,12 +7544,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -7630,12 +7632,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -7718,12 +7720,12 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -7806,12 +7808,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -7894,12 +7896,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -7982,12 +7984,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -8070,12 +8072,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -8158,12 +8160,12 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>DHARMAPURI</t>
+          <t>DARIPURI</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>ANDARA EKA Standard</t>
+          <t>BANDARA EKA Standard</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -8246,12 +8248,12 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -8334,12 +8336,12 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -8422,12 +8424,12 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>VETRA Standard</t>
+          <t>VESPA Standard</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -8510,12 +8512,12 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -8598,12 +8600,12 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>VASA Standard</t>
+          <t>VISA Standard</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -8686,12 +8688,12 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -8774,12 +8776,12 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -8862,12 +8864,12 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -8950,12 +8952,12 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -9038,12 +9040,12 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -9126,12 +9128,12 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -9214,12 +9216,12 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Akasha Standard</t>
+          <t>Akasih Standard</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -9302,12 +9304,12 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>NAVA Standard</t>
+          <t>NAWAR Standard</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -9390,12 +9392,12 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -9478,12 +9480,12 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>AVANYA S Standard</t>
+          <t>APANYA S Standard</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -9566,12 +9568,12 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -9654,12 +9656,12 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -9742,12 +9744,12 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -9830,12 +9832,12 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>AVANYA S Hook</t>
+          <t>APANYA S Hook</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -9918,12 +9920,12 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -10006,12 +10008,12 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Darmaraja Standard</t>
+          <t>Darmawisata Standard</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -10094,12 +10096,12 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>VETRA Standard</t>
+          <t>VESPA Standard</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -10176,6 +10178,358 @@
       <c r="R109" s="3" t="inlineStr">
         <is>
           <t>BILLBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="13" t="inlineStr">
+        <is>
+          <t>ASCOGRIYA</t>
+        </is>
+      </c>
+      <c r="B110" s="13" t="inlineStr">
+        <is>
+          <t>VESPA Standard</t>
+        </is>
+      </c>
+      <c r="C110" s="13" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D110" s="13" t="inlineStr">
+        <is>
+          <t>6 x 16</t>
+        </is>
+      </c>
+      <c r="E110" s="13" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="F110" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G110" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H110" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I110" s="13" t="inlineStr">
+        <is>
+          <t>29-Sep-26</t>
+        </is>
+      </c>
+      <c r="J110" s="13" t="inlineStr">
+        <is>
+          <t>BANDUNG</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>28</v>
+      </c>
+      <c r="L110" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M110" s="14" t="n">
+        <v>2.022</v>
+      </c>
+      <c r="N110" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="O110" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="P110" s="13" t="inlineStr">
+        <is>
+          <t>WIRASWASTA</t>
+        </is>
+      </c>
+      <c r="Q110" s="13" t="inlineStr">
+        <is>
+          <t>IN HOUSE</t>
+        </is>
+      </c>
+      <c r="R110" s="13" t="inlineStr">
+        <is>
+          <t>BILLBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="13" t="inlineStr">
+        <is>
+          <t>ASCOGRIYA</t>
+        </is>
+      </c>
+      <c r="B111" s="13" t="inlineStr">
+        <is>
+          <t>VESPA Standard</t>
+        </is>
+      </c>
+      <c r="C111" s="13" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D111" s="13" t="inlineStr">
+        <is>
+          <t>6 x 16</t>
+        </is>
+      </c>
+      <c r="E111" s="13" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="F111" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G111" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H111" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I111" s="13" t="inlineStr">
+        <is>
+          <t>29-Sep-26</t>
+        </is>
+      </c>
+      <c r="J111" s="13" t="inlineStr">
+        <is>
+          <t>BANDUNG</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>28</v>
+      </c>
+      <c r="L111" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M111" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="N111" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="O111" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="P111" s="13" t="inlineStr">
+        <is>
+          <t>WIRASWASTA</t>
+        </is>
+      </c>
+      <c r="Q111" s="13" t="inlineStr">
+        <is>
+          <t>IN HOUSE</t>
+        </is>
+      </c>
+      <c r="R111" s="13" t="inlineStr">
+        <is>
+          <t>BILLBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="13" t="inlineStr">
+        <is>
+          <t>PETROGRIYA</t>
+        </is>
+      </c>
+      <c r="B112" s="13" t="inlineStr">
+        <is>
+          <t>APANYA Hook</t>
+        </is>
+      </c>
+      <c r="C112" s="13" t="inlineStr">
+        <is>
+          <t>Hook</t>
+        </is>
+      </c>
+      <c r="D112" s="13" t="inlineStr">
+        <is>
+          <t>5 x 15</t>
+        </is>
+      </c>
+      <c r="E112" s="13" t="inlineStr">
+        <is>
+          <t>06/03</t>
+        </is>
+      </c>
+      <c r="F112" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G112" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H112" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I112" s="13" t="inlineStr">
+        <is>
+          <t>08-Sep-26</t>
+        </is>
+      </c>
+      <c r="J112" s="13" t="inlineStr">
+        <is>
+          <t>CIMAHI</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>34</v>
+      </c>
+      <c r="L112" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M112" s="14" t="n">
+        <v>1.333</v>
+      </c>
+      <c r="N112" s="13" t="inlineStr">
+        <is>
+          <t>KB 30x</t>
+        </is>
+      </c>
+      <c r="O112" s="13" t="inlineStr">
+        <is>
+          <t>Cash Bertahap</t>
+        </is>
+      </c>
+      <c r="P112" s="13" t="inlineStr">
+        <is>
+          <t>IBU RUMAH TANGGA</t>
+        </is>
+      </c>
+      <c r="Q112" s="13" t="inlineStr">
+        <is>
+          <t>RINA (DUMMY) - PROPERTI MANDIRI</t>
+        </is>
+      </c>
+      <c r="R112" s="13" t="inlineStr">
+        <is>
+          <t>AGENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="13" t="inlineStr">
+        <is>
+          <t>PETROGRIYA</t>
+        </is>
+      </c>
+      <c r="B113" s="13" t="inlineStr">
+        <is>
+          <t>APANYA Hook</t>
+        </is>
+      </c>
+      <c r="C113" s="13" t="inlineStr">
+        <is>
+          <t>Hook</t>
+        </is>
+      </c>
+      <c r="D113" s="13" t="inlineStr">
+        <is>
+          <t>5 x 15</t>
+        </is>
+      </c>
+      <c r="E113" s="13" t="inlineStr">
+        <is>
+          <t>06/03</t>
+        </is>
+      </c>
+      <c r="F113" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G113" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H113" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I113" s="13" t="inlineStr">
+        <is>
+          <t>08-Sep-26</t>
+        </is>
+      </c>
+      <c r="J113" s="13" t="inlineStr">
+        <is>
+          <t>CIMAHI</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>34</v>
+      </c>
+      <c r="L113" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M113" s="14" t="n">
+        <v>1.333</v>
+      </c>
+      <c r="N113" s="13" t="inlineStr">
+        <is>
+          <t>KB 30x</t>
+        </is>
+      </c>
+      <c r="O113" s="13" t="inlineStr">
+        <is>
+          <t>Cash Bertahap</t>
+        </is>
+      </c>
+      <c r="P113" s="13" t="inlineStr">
+        <is>
+          <t>IBU RUMAH TANGGA</t>
+        </is>
+      </c>
+      <c r="Q113" s="13" t="inlineStr">
+        <is>
+          <t>RINA (DUMMY) - PROPERTI MANDIRI</t>
+        </is>
+      </c>
+      <c r="R113" s="13" t="inlineStr">
+        <is>
+          <t>AGENT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Checkpoint 2 dengan nama samaran dan README ringkas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Y8Us56muFbCjBwSqpr5Hk
</commit_message>
<xml_diff>
--- a/REKAP_ALL_TIME_DUMMY.xlsx
+++ b/REKAP_ALL_TIME_DUMMY.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,6 +119,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -560,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R109"/>
+  <dimension ref="A1:R113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -678,12 +680,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -766,12 +768,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Darmaraja Standard</t>
+          <t>Darmawisata Standard</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -854,12 +856,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>LA PLAZA</t>
+          <t>UHUY PLAZA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>LP Standard</t>
+          <t>UHP Standard</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -942,12 +944,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>NP Standard</t>
+          <t>UP Standard</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1030,12 +1032,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1118,12 +1120,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>VETRA Standard</t>
+          <t>VESPA Standard</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1206,12 +1208,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>VASA Standard</t>
+          <t>VISA Standard</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1294,12 +1296,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Wanayasa Hook</t>
+          <t>Wanabisa Hook</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1382,12 +1384,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Hook</t>
+          <t>APEGEL S Hook</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1470,12 +1472,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1558,12 +1560,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1646,12 +1648,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1734,12 +1736,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>THE PLAZA</t>
+          <t>ESTHE PLAZA</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>TP Standard</t>
+          <t>EP Standard</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1822,12 +1824,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1910,12 +1912,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1998,12 +2000,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -2086,12 +2088,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DHARMAPURI</t>
+          <t>DARIPURI</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>ARUNA EKA Standard</t>
+          <t>AROMA EKA Standard</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -2174,12 +2176,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2262,12 +2264,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2350,12 +2352,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2438,12 +2440,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2526,12 +2528,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2614,12 +2616,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>NAVA Standard</t>
+          <t>NAWAR Standard</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2702,12 +2704,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2790,12 +2792,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2878,12 +2880,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>SVARA EKA Standard</t>
+          <t>SUARA EKA Standard</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2966,12 +2968,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -3054,12 +3056,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -3142,12 +3144,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -3230,12 +3232,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -3318,12 +3320,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -3406,12 +3408,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Akasha Hook</t>
+          <t>Akasih Hook</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -3494,12 +3496,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Darmaraja Standard</t>
+          <t>Darmawisata Standard</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3582,12 +3584,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -3670,12 +3672,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>NAVA Hook</t>
+          <t>NAWAR Hook</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3758,12 +3760,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>NP Standard</t>
+          <t>UP Standard</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -3846,12 +3848,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -3934,12 +3936,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LA PLAZA</t>
+          <t>UHUY PLAZA</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>LP Standard</t>
+          <t>UHP Standard</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -4022,12 +4024,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>NP Standard</t>
+          <t>UP Standard</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -4110,12 +4112,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -4198,12 +4200,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>SVARA EKA Hook</t>
+          <t>SUARA EKA Hook</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -4286,12 +4288,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>THE PLAZA</t>
+          <t>ESTHE PLAZA</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>TP Standard</t>
+          <t>EP Standard</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -4374,12 +4376,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Hook</t>
+          <t>APEGEL S Hook</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -4462,12 +4464,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Standard</t>
+          <t>AMBYAR TRI Standard</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -4550,12 +4552,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -4638,12 +4640,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -4726,12 +4728,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -4814,12 +4816,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>VETRA Hook</t>
+          <t>VESPA Hook</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -4902,12 +4904,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>SAGARA Hook</t>
+          <t>SEGERA Hook</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -4990,12 +4992,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Akasha Standard</t>
+          <t>Akasih Standard</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -5078,12 +5080,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Standard</t>
+          <t>AMBYAR TRI Standard</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -5166,12 +5168,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>VASA Standard</t>
+          <t>VISA Standard</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -5254,12 +5256,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>SVARA EKA Standard</t>
+          <t>SUARA EKA Standard</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -5342,12 +5344,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Standard</t>
+          <t>AMBYAR TRI Standard</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -5430,12 +5432,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>SAGARA Standard</t>
+          <t>SEGERA Standard</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -5518,12 +5520,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Standard</t>
+          <t>ARENA EKA Standard</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -5606,12 +5608,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -5694,12 +5696,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -5782,12 +5784,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -5870,12 +5872,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -5958,12 +5960,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>NEO PLAZA</t>
+          <t>UNO PLAZA</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>NP Hook</t>
+          <t>UP Hook</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -6046,12 +6048,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -6134,12 +6136,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Akasha Hook</t>
+          <t>Akasih Hook</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -6222,12 +6224,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Akasha Standard</t>
+          <t>Akasih Standard</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -6310,12 +6312,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>NAVA Standard</t>
+          <t>NAWAR Standard</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -6398,12 +6400,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -6486,12 +6488,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -6574,12 +6576,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>AMALA TRI Hook</t>
+          <t>AMBYAR TRI Hook</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -6662,12 +6664,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -6750,12 +6752,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Akasha Hook</t>
+          <t>Akasih Hook</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -6838,12 +6840,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Standard</t>
+          <t>ARENA EKA Standard</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -6926,12 +6928,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>NAVA Hook</t>
+          <t>NAWAR Hook</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -7014,12 +7016,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>SAGARA Standard</t>
+          <t>SEGERA Standard</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -7102,12 +7104,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -7190,12 +7192,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Hook</t>
+          <t>AMBYAR EKA Hook</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -7278,12 +7280,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -7366,12 +7368,12 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -7454,12 +7456,12 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>VETRA Hook</t>
+          <t>VESPA Hook</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -7542,12 +7544,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -7630,12 +7632,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -7718,12 +7720,12 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -7806,12 +7808,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -7894,12 +7896,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>SADYAGRIYA</t>
+          <t>SAYAGRIYA</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>AMALA EKA Standard</t>
+          <t>AMBYAR EKA Standard</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -7982,12 +7984,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -8070,12 +8072,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>GRAND CALYA Standard</t>
+          <t>GRAND CILOK Standard</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -8158,12 +8160,12 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>DHARMAPURI</t>
+          <t>DARIPURI</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>ANDARA EKA Standard</t>
+          <t>BANDARA EKA Standard</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -8246,12 +8248,12 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -8334,12 +8336,12 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Arsana Standard</t>
+          <t>Arisan Standard</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -8422,12 +8424,12 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>VETRA Standard</t>
+          <t>VESPA Standard</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -8510,12 +8512,12 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>BRAHMAPURI</t>
+          <t>KHRISNAPURI</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>ASKARA Standard</t>
+          <t>ASMARA Standard</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -8598,12 +8600,12 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>VASA Standard</t>
+          <t>VISA Standard</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -8686,12 +8688,12 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -8774,12 +8776,12 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ARUNAGRIYA</t>
+          <t>SERUGRIYA</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>SVARA DWI Standard</t>
+          <t>SUARA DWI Standard</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -8862,12 +8864,12 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -8950,12 +8952,12 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -9038,12 +9040,12 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -9126,12 +9128,12 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -9214,12 +9216,12 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>PADMAGRIYA</t>
+          <t>PASTIGRIYA</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Akasha Standard</t>
+          <t>Akasih Standard</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -9302,12 +9304,12 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>NARAGRIYA</t>
+          <t>CIKONENGRAYA</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>NAVA Standard</t>
+          <t>NAWAR Standard</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -9390,12 +9392,12 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Standard</t>
+          <t>APANYA Standard</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -9478,12 +9480,12 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>AVANYA S Standard</t>
+          <t>APANYA S Standard</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -9566,12 +9568,12 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>AVEGA S Standard</t>
+          <t>APEGEL S Standard</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -9654,12 +9656,12 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>AVANYA Hook</t>
+          <t>APANYA Hook</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -9742,12 +9744,12 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA</t>
+          <t>PETROGRIYA</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>AVEGA Standard</t>
+          <t>APEGEL Standard</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -9830,12 +9832,12 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>PATRAGRIYA SHIMIZU</t>
+          <t>JEPUNGRIYA</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>AVANYA S Hook</t>
+          <t>APANYA S Hook</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -9918,12 +9920,12 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>ARANA EKA Hook</t>
+          <t>ARENA EKA Hook</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -10006,12 +10008,12 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>ANAPURI</t>
+          <t>ENTEPURI</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Darmaraja Standard</t>
+          <t>Darmawisata Standard</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -10094,12 +10096,12 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>WANGSAGRIYA</t>
+          <t>ASCOGRIYA</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>VETRA Standard</t>
+          <t>VESPA Standard</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -10176,6 +10178,358 @@
       <c r="R109" s="3" t="inlineStr">
         <is>
           <t>BILLBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="13" t="inlineStr">
+        <is>
+          <t>ASCOGRIYA</t>
+        </is>
+      </c>
+      <c r="B110" s="13" t="inlineStr">
+        <is>
+          <t>VESPA Standard</t>
+        </is>
+      </c>
+      <c r="C110" s="13" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D110" s="13" t="inlineStr">
+        <is>
+          <t>6 x 16</t>
+        </is>
+      </c>
+      <c r="E110" s="13" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="F110" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G110" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H110" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I110" s="13" t="inlineStr">
+        <is>
+          <t>29-Sep-26</t>
+        </is>
+      </c>
+      <c r="J110" s="13" t="inlineStr">
+        <is>
+          <t>BANDUNG</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>28</v>
+      </c>
+      <c r="L110" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M110" s="14" t="n">
+        <v>2.022</v>
+      </c>
+      <c r="N110" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="O110" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="P110" s="13" t="inlineStr">
+        <is>
+          <t>WIRASWASTA</t>
+        </is>
+      </c>
+      <c r="Q110" s="13" t="inlineStr">
+        <is>
+          <t>IN HOUSE</t>
+        </is>
+      </c>
+      <c r="R110" s="13" t="inlineStr">
+        <is>
+          <t>BILLBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="13" t="inlineStr">
+        <is>
+          <t>ASCOGRIYA</t>
+        </is>
+      </c>
+      <c r="B111" s="13" t="inlineStr">
+        <is>
+          <t>VESPA Standard</t>
+        </is>
+      </c>
+      <c r="C111" s="13" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D111" s="13" t="inlineStr">
+        <is>
+          <t>6 x 16</t>
+        </is>
+      </c>
+      <c r="E111" s="13" t="inlineStr">
+        <is>
+          <t>06/08</t>
+        </is>
+      </c>
+      <c r="F111" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G111" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H111" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I111" s="13" t="inlineStr">
+        <is>
+          <t>29-Sep-26</t>
+        </is>
+      </c>
+      <c r="J111" s="13" t="inlineStr">
+        <is>
+          <t>BANDUNG</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>28</v>
+      </c>
+      <c r="L111" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M111" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="N111" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="O111" s="13" t="inlineStr">
+        <is>
+          <t>KPR</t>
+        </is>
+      </c>
+      <c r="P111" s="13" t="inlineStr">
+        <is>
+          <t>WIRASWASTA</t>
+        </is>
+      </c>
+      <c r="Q111" s="13" t="inlineStr">
+        <is>
+          <t>IN HOUSE</t>
+        </is>
+      </c>
+      <c r="R111" s="13" t="inlineStr">
+        <is>
+          <t>BILLBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="13" t="inlineStr">
+        <is>
+          <t>PETROGRIYA</t>
+        </is>
+      </c>
+      <c r="B112" s="13" t="inlineStr">
+        <is>
+          <t>APANYA Hook</t>
+        </is>
+      </c>
+      <c r="C112" s="13" t="inlineStr">
+        <is>
+          <t>Hook</t>
+        </is>
+      </c>
+      <c r="D112" s="13" t="inlineStr">
+        <is>
+          <t>5 x 15</t>
+        </is>
+      </c>
+      <c r="E112" s="13" t="inlineStr">
+        <is>
+          <t>06/03</t>
+        </is>
+      </c>
+      <c r="F112" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G112" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H112" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I112" s="13" t="inlineStr">
+        <is>
+          <t>08-Sep-26</t>
+        </is>
+      </c>
+      <c r="J112" s="13" t="inlineStr">
+        <is>
+          <t>CIMAHI</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>34</v>
+      </c>
+      <c r="L112" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M112" s="14" t="n">
+        <v>1.333</v>
+      </c>
+      <c r="N112" s="13" t="inlineStr">
+        <is>
+          <t>KB 30x</t>
+        </is>
+      </c>
+      <c r="O112" s="13" t="inlineStr">
+        <is>
+          <t>Cash Bertahap</t>
+        </is>
+      </c>
+      <c r="P112" s="13" t="inlineStr">
+        <is>
+          <t>IBU RUMAH TANGGA</t>
+        </is>
+      </c>
+      <c r="Q112" s="13" t="inlineStr">
+        <is>
+          <t>RINA (DUMMY) - PROPERTI MANDIRI</t>
+        </is>
+      </c>
+      <c r="R112" s="13" t="inlineStr">
+        <is>
+          <t>AGENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="13" t="inlineStr">
+        <is>
+          <t>PETROGRIYA</t>
+        </is>
+      </c>
+      <c r="B113" s="13" t="inlineStr">
+        <is>
+          <t>APANYA Hook</t>
+        </is>
+      </c>
+      <c r="C113" s="13" t="inlineStr">
+        <is>
+          <t>Hook</t>
+        </is>
+      </c>
+      <c r="D113" s="13" t="inlineStr">
+        <is>
+          <t>5 x 15</t>
+        </is>
+      </c>
+      <c r="E113" s="13" t="inlineStr">
+        <is>
+          <t>06/03</t>
+        </is>
+      </c>
+      <c r="F113" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G113" s="13" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="H113" s="13" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="I113" s="13" t="inlineStr">
+        <is>
+          <t>08-Sep-26</t>
+        </is>
+      </c>
+      <c r="J113" s="13" t="inlineStr">
+        <is>
+          <t>CIMAHI</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>34</v>
+      </c>
+      <c r="L113" s="13" t="inlineStr">
+        <is>
+          <t>PAKAI SENDIRI</t>
+        </is>
+      </c>
+      <c r="M113" s="14" t="n">
+        <v>1.333</v>
+      </c>
+      <c r="N113" s="13" t="inlineStr">
+        <is>
+          <t>KB 30x</t>
+        </is>
+      </c>
+      <c r="O113" s="13" t="inlineStr">
+        <is>
+          <t>Cash Bertahap</t>
+        </is>
+      </c>
+      <c r="P113" s="13" t="inlineStr">
+        <is>
+          <t>IBU RUMAH TANGGA</t>
+        </is>
+      </c>
+      <c r="Q113" s="13" t="inlineStr">
+        <is>
+          <t>RINA (DUMMY) - PROPERTI MANDIRI</t>
+        </is>
+      </c>
+      <c r="R113" s="13" t="inlineStr">
+        <is>
+          <t>AGENT</t>
         </is>
       </c>
     </row>

</xml_diff>